<commit_message>
feat: sync multi-arquivo urgencia (marco+abril), botao Sync, cache SAMU/Produtividade
</commit_message>
<xml_diff>
--- a/PowerBI/urgencia_tratado_validado.xlsx
+++ b/PowerBI/urgencia_tratado_validado.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Inovar Soluções\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183B36E5-3CD4-4E73-A8FC-545D8EDD1BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{963F71C0-C541-4E77-B28B-CF23C2FBB87A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23232" windowHeight="12432" firstSheet="7" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMO_EXECUTIVO" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
     <sheet name="CHECK_DIARIO_MAPA_UPAII" sheetId="12" r:id="rId12"/>
     <sheet name="SAMU" sheetId="13" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
@@ -1300,13 +1300,6 @@
     <t>META</t>
   </si>
   <si>
-    <t>ATENDIMENTO REALIZADO PELA USA TERRESTRE (COM ENVIO DA VIATURA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ATENDIMENTO DAS CHAMADAS RECEBIDAS PELA CENTRAL DE REGULAÇÃO DAS URGÊNCIAS COM ORIENTAÇÃO (SEM ENVIO DE VIATURA)
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">03.01.03.014-6 
 </t>
   </si>
@@ -1354,6 +1347,13 @@
   </si>
   <si>
     <t>TOTAL:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATENDIMENTO DAS CHAMADAS RECEBIDAS PELA CENTRAL DE REGULAÇÃO DAS URGÊNCIAS COM ORIENTAÇÃO (SEM ENVIO DE VIATURA) 148,5
+</t>
+  </si>
+  <si>
+    <t>ATENDIMENTO REALIZADO PELA USA TERRESTRE (COM ENVIO DA VIATURA)60,5</t>
   </si>
 </sst>
 </file>
@@ -7651,9 +7651,9 @@
         <v>421</v>
       </c>
     </row>
-    <row r="4" spans="1:37" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
-        <v>422</v>
+        <v>438</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>28</v>
@@ -7762,10 +7762,10 @@
     </row>
     <row r="5" spans="1:37" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
-        <v>423</v>
+        <v>437</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="C5" s="9">
         <v>6</v>
@@ -7875,10 +7875,10 @@
     </row>
     <row r="6" spans="1:37" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="13" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="C6" s="15">
         <v>3</v>
@@ -7984,10 +7984,10 @@
     </row>
     <row r="7" spans="1:37" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="13" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="C7" s="15">
         <v>0</v>
@@ -8093,10 +8093,10 @@
     </row>
     <row r="8" spans="1:37" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="18" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
       <c r="C8" s="20">
         <v>1</v>
@@ -8202,10 +8202,10 @@
     </row>
     <row r="9" spans="1:37" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="23" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="C9" s="25">
         <v>4</v>
@@ -8311,10 +8311,10 @@
     </row>
     <row r="10" spans="1:37" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="23" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="C10" s="25">
         <v>4</v>
@@ -8420,10 +8420,10 @@
     </row>
     <row r="11" spans="1:37" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="23" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="C11" s="25">
         <v>0</v>
@@ -8529,10 +8529,10 @@
     </row>
     <row r="12" spans="1:37" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="23" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B12" s="28" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="C12" s="25">
         <v>0</v>
@@ -8638,7 +8638,7 @@
     </row>
     <row r="13" spans="1:37" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="39" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="B13" s="40"/>
       <c r="C13" s="29">
@@ -8747,6 +8747,7 @@
     <mergeCell ref="A13:B13"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967294" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>